<commit_message>
Integrate NSMO horizon sensitivity into app and Excel
</commit_message>
<xml_diff>
--- a/apps/excel/templates/CreditAtlas-NSMO-Reference.xlsx
+++ b/apps/excel/templates/CreditAtlas-NSMO-Reference.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bat dau" sheetId="1" r:id="R33e31be7cf774220"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tu dien 587 truong" sheetId="2" r:id="Rde7df2364b554384"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nhan va category" sheetId="3" r:id="R410ca2f1d1804107"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage theo wave" sheetId="4" r:id="R11a648f6747c4ad4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="So sanh wording item" sheetId="5" r:id="R11654363fb5849e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bat dau" sheetId="1" r:id="R796fd279c43d45fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tu dien 587 truong" sheetId="2" r:id="R13df27298d0d4b05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nhan va category" sheetId="3" r:id="R5165920f2ba44ca7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage theo wave" sheetId="4" r:id="R71032f590c2b4b2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="So sanh wording item" sheetId="5" r:id="R013d95c906894ed1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do nhay horizon" sheetId="6" r:id="Rbecd38723c3d45d6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,6 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="#,##0"/>
+  </x:numFmts>
   <x:fonts count="4">
     <x:font>
       <x:sz val="11"/>
@@ -66,7 +70,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="16">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -101,6 +105,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -180,6 +187,23 @@
     <x:tableColumn id="7" name="Nhãn thang trả lời"/>
     <x:tableColumn id="8" name="Số gói questionnaire có wording"/>
     <x:tableColumn id="9" name="Đánh giá / giới hạn trend"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="NSMOReference5" displayName="NSMOReference5" ref="A1:H28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:H28"/>
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="Kỳ hạn (quý)"/>
+    <x:tableColumn id="2" name="Kỳ hạn xấp xỉ (tháng)"/>
+    <x:tableColumn id="3" name="Baseline C snapshots đủ follow-up"/>
+    <x:tableColumn id="4" name="Mortgage unique baseline"/>
+    <x:tableColumn id="5" name="Nhóm outcome"/>
+    <x:tableColumn id="6" name="Diễn giải / giới hạn"/>
+    <x:tableColumn id="7" name="Snapshot count (unweighted)"/>
+    <x:tableColumn id="8" name="Mortgage unique (không loại trừ)"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -386,7 +410,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>CreditAtlas · NSMO v7.0 reference workbook</x:v>
+        <x:v>CreditAtlas · NSMO v7.0 research workbook</x:v>
       </x:c>
       <x:c r="B1" s="4" t="str"/>
     </x:row>
@@ -395,7 +419,7 @@
         <x:v>Mục đích</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>Tra cứu codebook, nhãn category, coverage theo wave và ghi chú wording; workbook không chứa hồ sơ khoản vay.</x:v>
+        <x:v>Tra cứu codebook, category, coverage/wording theo wave và so sánh support quan sát được theo horizon; không chứa hồ sơ khoản vay.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
@@ -403,7 +427,7 @@
         <x:v>Nguồn</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>Bốn bảng metadata đã làm sạch trong docs/data; CSV gốc vẫn được dùng để app kiểm tra schema và tái tạo workbook.</x:v>
+        <x:v>Bốn bảng metadata trong docs/data và một bảng aggregate-only trong docs; PUF gốc được giữ riêng, receipt private ràng buộc SHA-256.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
@@ -411,7 +435,7 @@
         <x:v>Cách dùng</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>Bốn sheet dữ liệu là Excel Table: dùng bộ lọc ở tiêu đề, tìm mã biến/category và thêm ghi chú nội bộ ở cột mới.</x:v>
+        <x:v>Năm sheet dữ liệu là Excel Table có bộ lọc. Bảng horizon giữ snapshot counts và mortgage unique thành cột số để phân tích.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
@@ -440,10 +464,18 @@
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="7" t="str">
+        <x:v>Horizon sensitivity</x:v>
+      </x:c>
+      <x:c r="B8" s="9" t="str">
+        <x:v>So sánh 6/12/24 tháng từ baseline C; cohort không lồng nhau. Đây là support/censoring, không phải event rate hoặc PD.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="7" t="str">
         <x:v>Làm mới</x:v>
       </x:c>
-      <x:c r="B8" s="9" t="str">
-        <x:v>Chạy scripts/build_nsmo_reference_workbook.mjs với root project và đường dẫn output .xlsx.</x:v>
+      <x:c r="B9" s="9" t="str">
+        <x:v>Cập nhật CSV metadata/aggregate đã review, rồi chạy scripts/build_nsmo_reference_workbook.mjs với root project và output .xlsx.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -28114,7 +28146,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ff28c6759ca4d0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra393d3a8e6bc4a53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32289,7 +32321,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4fd8629bd2e4b1c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12b6bbaa93cc443e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41308,7 +41340,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc96dd1a38944b85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0be3612e9bd3469a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41601,7 +41633,757 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61068a07edc745d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R113bbb149a644e51"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="35" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="26" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="32" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="29" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="42" customHeight="1">
+      <x:c r="A1" s="13" t="str">
+        <x:v>Kỳ hạn (quý)</x:v>
+      </x:c>
+      <x:c r="B1" s="13" t="str">
+        <x:v>Kỳ hạn xấp xỉ (tháng)</x:v>
+      </x:c>
+      <x:c r="C1" s="13" t="str">
+        <x:v>Baseline C snapshots đủ follow-up</x:v>
+      </x:c>
+      <x:c r="D1" s="13" t="str">
+        <x:v>Mortgage unique baseline</x:v>
+      </x:c>
+      <x:c r="E1" s="13" t="str">
+        <x:v>Nhóm outcome</x:v>
+      </x:c>
+      <x:c r="F1" s="13" t="str">
+        <x:v>Diễn giải / giới hạn</x:v>
+      </x:c>
+      <x:c r="G1" s="13" t="str">
+        <x:v>Snapshot count (unweighted)</x:v>
+      </x:c>
+      <x:c r="H1" s="13" t="str">
+        <x:v>Mortgage unique (không loại trừ)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="42" customHeight="1">
+      <x:c r="A2" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B2" s="15" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C2" s="15" t="n">
+        <x:v>926331</x:v>
+      </x:c>
+      <x:c r="D2" s="15" t="n">
+        <x:v>61645</x:v>
+      </x:c>
+      <x:c r="E2" s="9" t="str">
+        <x:v>CENSOR_M</x:v>
+      </x:c>
+      <x:c r="F2" s="9" t="str">
+        <x:v>Censor quan sát: gap lịch sử (M)</x:v>
+      </x:c>
+      <x:c r="G2" s="15" t="n">
+        <x:v>661</x:v>
+      </x:c>
+      <x:c r="H2" s="15" t="n">
+        <x:v>394</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="42" customHeight="1">
+      <x:c r="A3" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="15" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C3" s="15" t="n">
+        <x:v>926331</x:v>
+      </x:c>
+      <x:c r="D3" s="15" t="n">
+        <x:v>61645</x:v>
+      </x:c>
+      <x:c r="E3" s="9" t="str">
+        <x:v>CENSOR_S</x:v>
+      </x:c>
+      <x:c r="F3" s="9" t="str">
+        <x:v>Censor quan sát: servicer suppression (S)</x:v>
+      </x:c>
+      <x:c r="G3" s="15" t="n">
+        <x:v>2776</x:v>
+      </x:c>
+      <x:c r="H3" s="15" t="n">
+        <x:v>1332</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="42" customHeight="1">
+      <x:c r="A4" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B4" s="15" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C4" s="15" t="n">
+        <x:v>926331</x:v>
+      </x:c>
+      <x:c r="D4" s="15" t="n">
+        <x:v>61645</x:v>
+      </x:c>
+      <x:c r="E4" s="9" t="str">
+        <x:v>90PLUS</x:v>
+      </x:c>
+      <x:c r="F4" s="9" t="str">
+        <x:v>Quan sát 90+ ngày trễ (mã 3–6)</x:v>
+      </x:c>
+      <x:c r="G4" s="15" t="n">
+        <x:v>964</x:v>
+      </x:c>
+      <x:c r="H4" s="15" t="n">
+        <x:v>623</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="42" customHeight="1">
+      <x:c r="A5" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="15" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C5" s="15" t="n">
+        <x:v>926331</x:v>
+      </x:c>
+      <x:c r="D5" s="15" t="n">
+        <x:v>61645</x:v>
+      </x:c>
+      <x:c r="E5" s="9" t="str">
+        <x:v>NO_90PLUS</x:v>
+      </x:c>
+      <x:c r="F5" s="9" t="str">
+        <x:v>Không quan sát 90+ trong các snapshot kỳ hạn này; không chứng minh lịch sử hoàn toàn không có event</x:v>
+      </x:c>
+      <x:c r="G5" s="15" t="n">
+        <x:v>854164</x:v>
+      </x:c>
+      <x:c r="H5" s="15" t="n">
+        <x:v>58387</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="15" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C6" s="15" t="n">
+        <x:v>926331</x:v>
+      </x:c>
+      <x:c r="D6" s="15" t="n">
+        <x:v>61645</x:v>
+      </x:c>
+      <x:c r="E6" s="9" t="str">
+        <x:v>OTHER_7</x:v>
+      </x:c>
+      <x:c r="F6" s="9" t="str">
+        <x:v>Trạng thái cạnh tranh: bankruptcy (7)</x:v>
+      </x:c>
+      <x:c r="G6" s="15" t="n">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="H6" s="15" t="n">
+        <x:v>48</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B7" s="15" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C7" s="15" t="n">
+        <x:v>926331</x:v>
+      </x:c>
+      <x:c r="D7" s="15" t="n">
+        <x:v>61645</x:v>
+      </x:c>
+      <x:c r="E7" s="9" t="str">
+        <x:v>OTHER_8</x:v>
+      </x:c>
+      <x:c r="F7" s="9" t="str">
+        <x:v>Trạng thái cạnh tranh: foreclosure/distressed (8)</x:v>
+      </x:c>
+      <x:c r="G7" s="15" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H7" s="15" t="n">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B8" s="15" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C8" s="15" t="n">
+        <x:v>926331</x:v>
+      </x:c>
+      <x:c r="D8" s="15" t="n">
+        <x:v>61645</x:v>
+      </x:c>
+      <x:c r="E8" s="9" t="str">
+        <x:v>OTHER_9</x:v>
+      </x:c>
+      <x:c r="F8" s="9" t="str">
+        <x:v>Trạng thái cạnh tranh: giải quyết/charge-off khác (9)</x:v>
+      </x:c>
+      <x:c r="G8" s="15" t="n">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="H8" s="15" t="n">
+        <x:v>62</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B9" s="15" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C9" s="15" t="n">
+        <x:v>926331</x:v>
+      </x:c>
+      <x:c r="D9" s="15" t="n">
+        <x:v>61645</x:v>
+      </x:c>
+      <x:c r="E9" s="9" t="str">
+        <x:v>CLOSE_PRE</x:v>
+      </x:c>
+      <x:c r="F9" s="9" t="str">
+        <x:v>Kết thúc trước snapshot kế tiếp; nguyên nhân không rõ</x:v>
+      </x:c>
+      <x:c r="G9" s="15" t="n">
+        <x:v>44695</x:v>
+      </x:c>
+      <x:c r="H9" s="15" t="n">
+        <x:v>22920</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="42" customHeight="1">
+      <x:c r="A10" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B10" s="15" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C10" s="15" t="n">
+        <x:v>926331</x:v>
+      </x:c>
+      <x:c r="D10" s="15" t="n">
+        <x:v>61645</x:v>
+      </x:c>
+      <x:c r="E10" s="9" t="str">
+        <x:v>CLOSE_TIED</x:v>
+      </x:c>
+      <x:c r="F10" s="9" t="str">
+        <x:v>Đóng cùng tháng snapshot; thứ tự không xác định</x:v>
+      </x:c>
+      <x:c r="G10" s="15" t="n">
+        <x:v>22849</x:v>
+      </x:c>
+      <x:c r="H10" s="15" t="n">
+        <x:v>11769</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="42" customHeight="1">
+      <x:c r="A11" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B11" s="15" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C11" s="15" t="n">
+        <x:v>872888</x:v>
+      </x:c>
+      <x:c r="D11" s="15" t="n">
+        <x:v>59703</x:v>
+      </x:c>
+      <x:c r="E11" s="9" t="str">
+        <x:v>CENSOR_M</x:v>
+      </x:c>
+      <x:c r="F11" s="9" t="str">
+        <x:v>Censor quan sát: gap lịch sử (M)</x:v>
+      </x:c>
+      <x:c r="G11" s="15" t="n">
+        <x:v>1067</x:v>
+      </x:c>
+      <x:c r="H11" s="15" t="n">
+        <x:v>387</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="42" customHeight="1">
+      <x:c r="A12" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B12" s="15" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C12" s="15" t="n">
+        <x:v>872888</x:v>
+      </x:c>
+      <x:c r="D12" s="15" t="n">
+        <x:v>59703</x:v>
+      </x:c>
+      <x:c r="E12" s="9" t="str">
+        <x:v>CENSOR_S</x:v>
+      </x:c>
+      <x:c r="F12" s="9" t="str">
+        <x:v>Censor quan sát: servicer suppression (S)</x:v>
+      </x:c>
+      <x:c r="G12" s="15" t="n">
+        <x:v>5129</x:v>
+      </x:c>
+      <x:c r="H12" s="15" t="n">
+        <x:v>1360</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="42" customHeight="1">
+      <x:c r="A13" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B13" s="15" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C13" s="15" t="n">
+        <x:v>872888</x:v>
+      </x:c>
+      <x:c r="D13" s="15" t="n">
+        <x:v>59703</x:v>
+      </x:c>
+      <x:c r="E13" s="9" t="str">
+        <x:v>90PLUS</x:v>
+      </x:c>
+      <x:c r="F13" s="9" t="str">
+        <x:v>Quan sát 90+ ngày trễ (mã 3–6)</x:v>
+      </x:c>
+      <x:c r="G13" s="15" t="n">
+        <x:v>2174</x:v>
+      </x:c>
+      <x:c r="H13" s="15" t="n">
+        <x:v>753</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="42" customHeight="1">
+      <x:c r="A14" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B14" s="15" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C14" s="15" t="n">
+        <x:v>872888</x:v>
+      </x:c>
+      <x:c r="D14" s="15" t="n">
+        <x:v>59703</x:v>
+      </x:c>
+      <x:c r="E14" s="9" t="str">
+        <x:v>NO_90PLUS</x:v>
+      </x:c>
+      <x:c r="F14" s="9" t="str">
+        <x:v>Không quan sát 90+ trong các snapshot kỳ hạn này; không chứng minh lịch sử hoàn toàn không có event</x:v>
+      </x:c>
+      <x:c r="G14" s="15" t="n">
+        <x:v>738773</x:v>
+      </x:c>
+      <x:c r="H14" s="15" t="n">
+        <x:v>52110</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="42" customHeight="1">
+      <x:c r="A15" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B15" s="15" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C15" s="15" t="n">
+        <x:v>872888</x:v>
+      </x:c>
+      <x:c r="D15" s="15" t="n">
+        <x:v>59703</x:v>
+      </x:c>
+      <x:c r="E15" s="9" t="str">
+        <x:v>OTHER_7</x:v>
+      </x:c>
+      <x:c r="F15" s="9" t="str">
+        <x:v>Trạng thái cạnh tranh: bankruptcy (7)</x:v>
+      </x:c>
+      <x:c r="G15" s="15" t="n">
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="H15" s="15" t="n">
+        <x:v>50</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="42" customHeight="1">
+      <x:c r="A16" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B16" s="15" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C16" s="15" t="n">
+        <x:v>872888</x:v>
+      </x:c>
+      <x:c r="D16" s="15" t="n">
+        <x:v>59703</x:v>
+      </x:c>
+      <x:c r="E16" s="9" t="str">
+        <x:v>OTHER_8</x:v>
+      </x:c>
+      <x:c r="F16" s="9" t="str">
+        <x:v>Trạng thái cạnh tranh: foreclosure/distressed (8)</x:v>
+      </x:c>
+      <x:c r="G16" s="15" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="H16" s="15" t="n">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="42" customHeight="1">
+      <x:c r="A17" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B17" s="15" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C17" s="15" t="n">
+        <x:v>872888</x:v>
+      </x:c>
+      <x:c r="D17" s="15" t="n">
+        <x:v>59703</x:v>
+      </x:c>
+      <x:c r="E17" s="9" t="str">
+        <x:v>OTHER_9</x:v>
+      </x:c>
+      <x:c r="F17" s="9" t="str">
+        <x:v>Trạng thái cạnh tranh: giải quyết/charge-off khác (9)</x:v>
+      </x:c>
+      <x:c r="G17" s="15" t="n">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="H17" s="15" t="n">
+        <x:v>63</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="42" customHeight="1">
+      <x:c r="A18" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B18" s="15" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C18" s="15" t="n">
+        <x:v>872888</x:v>
+      </x:c>
+      <x:c r="D18" s="15" t="n">
+        <x:v>59703</x:v>
+      </x:c>
+      <x:c r="E18" s="9" t="str">
+        <x:v>CLOSE_PRE</x:v>
+      </x:c>
+      <x:c r="F18" s="9" t="str">
+        <x:v>Kết thúc trước snapshot kế tiếp; nguyên nhân không rõ</x:v>
+      </x:c>
+      <x:c r="G18" s="15" t="n">
+        <x:v>83092</x:v>
+      </x:c>
+      <x:c r="H18" s="15" t="n">
+        <x:v>22843</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="42" customHeight="1">
+      <x:c r="A19" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B19" s="15" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C19" s="15" t="n">
+        <x:v>872888</x:v>
+      </x:c>
+      <x:c r="D19" s="15" t="n">
+        <x:v>59703</x:v>
+      </x:c>
+      <x:c r="E19" s="9" t="str">
+        <x:v>CLOSE_TIED</x:v>
+      </x:c>
+      <x:c r="F19" s="9" t="str">
+        <x:v>Đóng cùng tháng snapshot; thứ tự không xác định</x:v>
+      </x:c>
+      <x:c r="G19" s="15" t="n">
+        <x:v>42236</x:v>
+      </x:c>
+      <x:c r="H19" s="15" t="n">
+        <x:v>11749</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="42" customHeight="1">
+      <x:c r="A20" s="15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B20" s="15" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C20" s="15" t="n">
+        <x:v>770257</x:v>
+      </x:c>
+      <x:c r="D20" s="15" t="n">
+        <x:v>55701</x:v>
+      </x:c>
+      <x:c r="E20" s="9" t="str">
+        <x:v>CENSOR_M</x:v>
+      </x:c>
+      <x:c r="F20" s="9" t="str">
+        <x:v>Censor quan sát: gap lịch sử (M)</x:v>
+      </x:c>
+      <x:c r="G20" s="15" t="n">
+        <x:v>1476</x:v>
+      </x:c>
+      <x:c r="H20" s="15" t="n">
+        <x:v>360</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="42" customHeight="1">
+      <x:c r="A21" s="15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B21" s="15" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C21" s="15" t="n">
+        <x:v>770257</x:v>
+      </x:c>
+      <x:c r="D21" s="15" t="n">
+        <x:v>55701</x:v>
+      </x:c>
+      <x:c r="E21" s="9" t="str">
+        <x:v>CENSOR_S</x:v>
+      </x:c>
+      <x:c r="F21" s="9" t="str">
+        <x:v>Censor quan sát: servicer suppression (S)</x:v>
+      </x:c>
+      <x:c r="G21" s="15" t="n">
+        <x:v>8461</x:v>
+      </x:c>
+      <x:c r="H21" s="15" t="n">
+        <x:v>1331</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="42" customHeight="1">
+      <x:c r="A22" s="15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B22" s="15" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C22" s="15" t="n">
+        <x:v>770257</x:v>
+      </x:c>
+      <x:c r="D22" s="15" t="n">
+        <x:v>55701</x:v>
+      </x:c>
+      <x:c r="E22" s="9" t="str">
+        <x:v>90PLUS</x:v>
+      </x:c>
+      <x:c r="F22" s="9" t="str">
+        <x:v>Quan sát 90+ ngày trễ (mã 3–6)</x:v>
+      </x:c>
+      <x:c r="G22" s="15" t="n">
+        <x:v>3683</x:v>
+      </x:c>
+      <x:c r="H22" s="15" t="n">
+        <x:v>735</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="42" customHeight="1">
+      <x:c r="A23" s="15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B23" s="15" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C23" s="15" t="n">
+        <x:v>770257</x:v>
+      </x:c>
+      <x:c r="D23" s="15" t="n">
+        <x:v>55701</x:v>
+      </x:c>
+      <x:c r="E23" s="9" t="str">
+        <x:v>NO_90PLUS</x:v>
+      </x:c>
+      <x:c r="F23" s="9" t="str">
+        <x:v>Không quan sát 90+ trong các snapshot kỳ hạn này; không chứng minh lịch sử hoàn toàn không có event</x:v>
+      </x:c>
+      <x:c r="G23" s="15" t="n">
+        <x:v>544419</x:v>
+      </x:c>
+      <x:c r="H23" s="15" t="n">
+        <x:v>41635</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="42" customHeight="1">
+      <x:c r="A24" s="15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B24" s="15" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C24" s="15" t="n">
+        <x:v>770257</x:v>
+      </x:c>
+      <x:c r="D24" s="15" t="n">
+        <x:v>55701</x:v>
+      </x:c>
+      <x:c r="E24" s="9" t="str">
+        <x:v>OTHER_7</x:v>
+      </x:c>
+      <x:c r="F24" s="9" t="str">
+        <x:v>Trạng thái cạnh tranh: bankruptcy (7)</x:v>
+      </x:c>
+      <x:c r="G24" s="15" t="n">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="H24" s="15" t="n">
+        <x:v>50</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="42" customHeight="1">
+      <x:c r="A25" s="15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B25" s="15" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C25" s="15" t="n">
+        <x:v>770257</x:v>
+      </x:c>
+      <x:c r="D25" s="15" t="n">
+        <x:v>55701</x:v>
+      </x:c>
+      <x:c r="E25" s="9" t="str">
+        <x:v>OTHER_8</x:v>
+      </x:c>
+      <x:c r="F25" s="9" t="str">
+        <x:v>Trạng thái cạnh tranh: foreclosure/distressed (8)</x:v>
+      </x:c>
+      <x:c r="G25" s="15" t="n">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="H25" s="15" t="n">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="42" customHeight="1">
+      <x:c r="A26" s="15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B26" s="15" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C26" s="15" t="n">
+        <x:v>770257</x:v>
+      </x:c>
+      <x:c r="D26" s="15" t="n">
+        <x:v>55701</x:v>
+      </x:c>
+      <x:c r="E26" s="9" t="str">
+        <x:v>OTHER_9</x:v>
+      </x:c>
+      <x:c r="F26" s="9" t="str">
+        <x:v>Trạng thái cạnh tranh: giải quyết/charge-off khác (9)</x:v>
+      </x:c>
+      <x:c r="G26" s="15" t="n">
+        <x:v>363</x:v>
+      </x:c>
+      <x:c r="H26" s="15" t="n">
+        <x:v>62</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="42" customHeight="1">
+      <x:c r="A27" s="15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B27" s="15" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C27" s="15" t="n">
+        <x:v>770257</x:v>
+      </x:c>
+      <x:c r="D27" s="15" t="n">
+        <x:v>55701</x:v>
+      </x:c>
+      <x:c r="E27" s="9" t="str">
+        <x:v>CLOSE_PRE</x:v>
+      </x:c>
+      <x:c r="F27" s="9" t="str">
+        <x:v>Kết thúc trước snapshot kế tiếp; nguyên nhân không rõ</x:v>
+      </x:c>
+      <x:c r="G27" s="15" t="n">
+        <x:v>140280</x:v>
+      </x:c>
+      <x:c r="H27" s="15" t="n">
+        <x:v>22324</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="42" customHeight="1">
+      <x:c r="A28" s="15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B28" s="15" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C28" s="15" t="n">
+        <x:v>770257</x:v>
+      </x:c>
+      <x:c r="D28" s="15" t="n">
+        <x:v>55701</x:v>
+      </x:c>
+      <x:c r="E28" s="9" t="str">
+        <x:v>CLOSE_TIED</x:v>
+      </x:c>
+      <x:c r="F28" s="9" t="str">
+        <x:v>Đóng cùng tháng snapshot; thứ tự không xác định</x:v>
+      </x:c>
+      <x:c r="G28" s="15" t="n">
+        <x:v>71229</x:v>
+      </x:c>
+      <x:c r="H28" s="15" t="n">
+        <x:v>11514</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc65ea100c11c4b94"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Clarify NSMO imputed-value coverage
</commit_message>
<xml_diff>
--- a/apps/excel/templates/CreditAtlas-NSMO-Reference.xlsx
+++ b/apps/excel/templates/CreditAtlas-NSMO-Reference.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bat dau" sheetId="1" r:id="R699560f88b3948e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tu dien 587 truong" sheetId="2" r:id="Rb39d65d7a4cb41bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nhan va category" sheetId="3" r:id="Rc60424dbca374574"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage theo wave" sheetId="4" r:id="Rb3ce32c95ca44f86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="So sanh wording item" sheetId="5" r:id="Rbdfd8249c3424edf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do nhay horizon" sheetId="6" r:id="R103eab3f78c74763"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bat dau" sheetId="1" r:id="R4315da49c8484ad3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tu dien 587 truong" sheetId="2" r:id="R7e4489bfcd17416b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nhan va category" sheetId="3" r:id="R6a106bb7e7cd4138"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage theo wave" sheetId="4" r:id="R7747393c27de4c96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="So sanh wording item" sheetId="5" r:id="R7b4903d88ed04de4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do nhay horizon" sheetId="6" r:id="Rf65e52121bc54de1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -163,7 +163,7 @@
     <x:tableColumn id="3" name="SAS format"/>
     <x:tableColumn id="4" name="Mã câu hỏi"/>
     <x:tableColumn id="5" name="Cờ biến thể codebook"/>
-    <x:tableColumn id="6" name="Wave có phản hồi quan sát"/>
+    <x:tableColumn id="6" name="Wave có giá trị PUF không thiếu (có thể đã impute)"/>
     <x:tableColumn id="7" name="Wave hoàn toàn không được hỏi (-3)"/>
     <x:tableColumn id="8" name="Wave được hỏi một phần (-3)"/>
     <x:tableColumn id="9" name="Wave không áp dụng (-2)"/>
@@ -180,7 +180,7 @@
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Tên cột CSV (giữ nguyên)"/>
     <x:tableColumn id="2" name="Nhãn SAS / câu hỏi"/>
-    <x:tableColumn id="3" name="Wave có phản hồi quan sát"/>
+    <x:tableColumn id="3" name="Wave có giá trị PUF không thiếu (có thể đã impute)"/>
     <x:tableColumn id="4" name="Wave không được hỏi"/>
     <x:tableColumn id="5" name="Mã câu hỏi"/>
     <x:tableColumn id="6" name="SAS format"/>
@@ -422,7 +422,7 @@
         <x:v>Mục đích</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>Tra cứu codebook, category, coverage/wording theo wave và so sánh support quan sát được theo horizon; không chứa hồ sơ khoản vay.</x:v>
+        <x:v>Tra cứu codebook, category, coverage/wording theo wave và so sánh support theo horizon; không chứa hồ sơ khoản vay.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
@@ -454,7 +454,7 @@
         <x:v>Coverage</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>Phản ánh availability/mã quan sát theo wave; không tự chứng minh cùng cách đo hoặc đủ điều kiện làm predictor.</x:v>
+        <x:v>Wave coverage đếm giá trị X không thiếu trong PUF, không xác nhận borrower đã trực tiếp trả lời: FHFA có thể impute giá trị thiếu vào biến X. PUF công khai không có cờ J theo từng item để nhận diện imputation; biến Z chỉ ghi nhận việc trả lời cho một số câu hỏi được chọn. Vì vậy không dùng các số đếm này làm response rate.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
@@ -28149,7 +28149,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb93db4476b7f4210"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcefe497a266e4998"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32324,7 +32324,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0497855d2164e1a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R304732ec89a44173"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32338,7 +32338,7 @@
     <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="27" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="52" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="36" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="29" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="25" hidden="0" customWidth="1"/>
@@ -32363,7 +32363,7 @@
         <x:v>Cờ biến thể codebook</x:v>
       </x:c>
       <x:c r="F1" s="13" t="str">
-        <x:v>Wave có phản hồi quan sát</x:v>
+        <x:v>Wave có giá trị PUF không thiếu (có thể đã impute)</x:v>
       </x:c>
       <x:c r="G1" s="13" t="str">
         <x:v>Wave hoàn toàn không được hỏi (-3)</x:v>
@@ -32405,7 +32405,7 @@
       <x:c r="I2" s="9" t="str"/>
       <x:c r="J2" s="9" t="str"/>
       <x:c r="K2" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -32432,7 +32432,7 @@
       <x:c r="I3" s="9" t="str"/>
       <x:c r="J3" s="9" t="str"/>
       <x:c r="K3" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -32459,7 +32459,7 @@
       <x:c r="I4" s="9" t="str"/>
       <x:c r="J4" s="9" t="str"/>
       <x:c r="K4" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -32486,7 +32486,7 @@
       <x:c r="I5" s="9" t="str"/>
       <x:c r="J5" s="9" t="str"/>
       <x:c r="K5" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -32511,7 +32511,7 @@
       <x:c r="I6" s="9" t="str"/>
       <x:c r="J6" s="9" t="str"/>
       <x:c r="K6" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -32538,7 +32538,7 @@
       <x:c r="I7" s="9" t="str"/>
       <x:c r="J7" s="9" t="str"/>
       <x:c r="K7" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -32565,7 +32565,7 @@
       <x:c r="I8" s="9" t="str"/>
       <x:c r="J8" s="9" t="str"/>
       <x:c r="K8" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -32592,7 +32592,7 @@
       <x:c r="I9" s="9" t="str"/>
       <x:c r="J9" s="9" t="str"/>
       <x:c r="K9" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -32619,7 +32619,7 @@
       <x:c r="I10" s="9" t="str"/>
       <x:c r="J10" s="9" t="str"/>
       <x:c r="K10" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -32646,7 +32646,7 @@
       <x:c r="I11" s="9" t="str"/>
       <x:c r="J11" s="9" t="str"/>
       <x:c r="K11" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -32671,7 +32671,7 @@
       <x:c r="I12" s="9" t="str"/>
       <x:c r="J12" s="9" t="str"/>
       <x:c r="K12" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -32698,7 +32698,7 @@
       <x:c r="I13" s="9" t="str"/>
       <x:c r="J13" s="9" t="str"/>
       <x:c r="K13" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -32725,7 +32725,7 @@
       <x:c r="I14" s="9" t="str"/>
       <x:c r="J14" s="9" t="str"/>
       <x:c r="K14" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -32752,7 +32752,7 @@
       <x:c r="I15" s="9" t="str"/>
       <x:c r="J15" s="9" t="str"/>
       <x:c r="K15" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -32781,7 +32781,7 @@
       <x:c r="I16" s="9" t="str"/>
       <x:c r="J16" s="9" t="str"/>
       <x:c r="K16" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -32808,7 +32808,7 @@
       <x:c r="I17" s="9" t="str"/>
       <x:c r="J17" s="9" t="str"/>
       <x:c r="K17" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -32835,7 +32835,7 @@
       <x:c r="I18" s="9" t="str"/>
       <x:c r="J18" s="9" t="str"/>
       <x:c r="K18" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -32860,7 +32860,7 @@
       <x:c r="I19" s="9" t="str"/>
       <x:c r="J19" s="9" t="str"/>
       <x:c r="K19" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -32887,7 +32887,7 @@
       <x:c r="I20" s="9" t="str"/>
       <x:c r="J20" s="9" t="str"/>
       <x:c r="K20" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -32912,7 +32912,7 @@
       <x:c r="I21" s="9" t="str"/>
       <x:c r="J21" s="9" t="str"/>
       <x:c r="K21" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -32939,7 +32939,7 @@
       <x:c r="I22" s="9" t="str"/>
       <x:c r="J22" s="9" t="str"/>
       <x:c r="K22" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -32966,7 +32966,7 @@
       <x:c r="I23" s="9" t="str"/>
       <x:c r="J23" s="9" t="str"/>
       <x:c r="K23" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -32995,7 +32995,7 @@
       </x:c>
       <x:c r="J24" s="9" t="str"/>
       <x:c r="K24" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -33024,7 +33024,7 @@
       </x:c>
       <x:c r="J25" s="9" t="str"/>
       <x:c r="K25" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -33053,7 +33053,7 @@
       </x:c>
       <x:c r="J26" s="9" t="str"/>
       <x:c r="K26" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -33080,7 +33080,7 @@
       </x:c>
       <x:c r="J27" s="9" t="str"/>
       <x:c r="K27" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -33109,7 +33109,7 @@
       <x:c r="I28" s="9" t="str"/>
       <x:c r="J28" s="9" t="str"/>
       <x:c r="K28" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -33138,7 +33138,7 @@
       <x:c r="I29" s="9" t="str"/>
       <x:c r="J29" s="9" t="str"/>
       <x:c r="K29" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -33165,7 +33165,7 @@
       <x:c r="I30" s="9" t="str"/>
       <x:c r="J30" s="9" t="str"/>
       <x:c r="K30" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -33194,7 +33194,7 @@
       <x:c r="I31" s="9" t="str"/>
       <x:c r="J31" s="9" t="str"/>
       <x:c r="K31" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -33223,7 +33223,7 @@
       <x:c r="I32" s="9" t="str"/>
       <x:c r="J32" s="9" t="str"/>
       <x:c r="K32" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -33252,7 +33252,7 @@
       <x:c r="I33" s="9" t="str"/>
       <x:c r="J33" s="9" t="str"/>
       <x:c r="K33" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -33281,7 +33281,7 @@
       <x:c r="I34" s="9" t="str"/>
       <x:c r="J34" s="9" t="str"/>
       <x:c r="K34" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -33308,7 +33308,7 @@
       <x:c r="I35" s="9" t="str"/>
       <x:c r="J35" s="9" t="str"/>
       <x:c r="K35" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -33337,7 +33337,7 @@
       <x:c r="I36" s="9" t="str"/>
       <x:c r="J36" s="9" t="str"/>
       <x:c r="K36" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -33366,7 +33366,7 @@
       <x:c r="I37" s="9" t="str"/>
       <x:c r="J37" s="9" t="str"/>
       <x:c r="K37" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -33395,7 +33395,7 @@
       <x:c r="I38" s="9" t="str"/>
       <x:c r="J38" s="9" t="str"/>
       <x:c r="K38" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -33424,7 +33424,7 @@
       <x:c r="I39" s="9" t="str"/>
       <x:c r="J39" s="9" t="str"/>
       <x:c r="K39" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -33453,7 +33453,7 @@
       <x:c r="I40" s="9" t="str"/>
       <x:c r="J40" s="9" t="str"/>
       <x:c r="K40" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -33480,7 +33480,7 @@
       <x:c r="I41" s="9" t="str"/>
       <x:c r="J41" s="9" t="str"/>
       <x:c r="K41" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -33509,7 +33509,7 @@
       <x:c r="I42" s="9" t="str"/>
       <x:c r="J42" s="9" t="str"/>
       <x:c r="K42" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -33538,7 +33538,7 @@
       <x:c r="I43" s="9" t="str"/>
       <x:c r="J43" s="9" t="str"/>
       <x:c r="K43" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -33567,7 +33567,7 @@
       <x:c r="I44" s="9" t="str"/>
       <x:c r="J44" s="9" t="str"/>
       <x:c r="K44" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -33596,7 +33596,7 @@
       <x:c r="I45" s="9" t="str"/>
       <x:c r="J45" s="9" t="str"/>
       <x:c r="K45" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -33625,7 +33625,7 @@
       <x:c r="I46" s="9" t="str"/>
       <x:c r="J46" s="9" t="str"/>
       <x:c r="K46" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -33652,7 +33652,7 @@
       <x:c r="I47" s="9" t="str"/>
       <x:c r="J47" s="9" t="str"/>
       <x:c r="K47" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -33679,7 +33679,7 @@
       <x:c r="I48" s="9" t="str"/>
       <x:c r="J48" s="9" t="str"/>
       <x:c r="K48" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -33708,7 +33708,7 @@
       </x:c>
       <x:c r="J49" s="9" t="str"/>
       <x:c r="K49" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -33737,7 +33737,7 @@
       <x:c r="I50" s="9" t="str"/>
       <x:c r="J50" s="9" t="str"/>
       <x:c r="K50" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -33766,7 +33766,7 @@
       <x:c r="I51" s="9" t="str"/>
       <x:c r="J51" s="9" t="str"/>
       <x:c r="K51" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -33795,7 +33795,7 @@
       <x:c r="I52" s="9" t="str"/>
       <x:c r="J52" s="9" t="str"/>
       <x:c r="K52" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -33824,7 +33824,7 @@
       <x:c r="I53" s="9" t="str"/>
       <x:c r="J53" s="9" t="str"/>
       <x:c r="K53" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -33853,7 +33853,7 @@
       <x:c r="I54" s="9" t="str"/>
       <x:c r="J54" s="9" t="str"/>
       <x:c r="K54" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -33882,7 +33882,7 @@
       <x:c r="I55" s="9" t="str"/>
       <x:c r="J55" s="9" t="str"/>
       <x:c r="K55" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -33909,7 +33909,7 @@
       <x:c r="I56" s="9" t="str"/>
       <x:c r="J56" s="9" t="str"/>
       <x:c r="K56" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -33938,7 +33938,7 @@
       <x:c r="I57" s="9" t="str"/>
       <x:c r="J57" s="9" t="str"/>
       <x:c r="K57" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -33967,7 +33967,7 @@
       <x:c r="I58" s="9" t="str"/>
       <x:c r="J58" s="9" t="str"/>
       <x:c r="K58" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -33996,7 +33996,7 @@
       <x:c r="I59" s="9" t="str"/>
       <x:c r="J59" s="9" t="str"/>
       <x:c r="K59" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -34025,7 +34025,7 @@
       <x:c r="I60" s="9" t="str"/>
       <x:c r="J60" s="9" t="str"/>
       <x:c r="K60" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -34054,7 +34054,7 @@
       <x:c r="I61" s="9" t="str"/>
       <x:c r="J61" s="9" t="str"/>
       <x:c r="K61" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -34083,7 +34083,7 @@
       <x:c r="I62" s="9" t="str"/>
       <x:c r="J62" s="9" t="str"/>
       <x:c r="K62" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -34110,7 +34110,7 @@
       <x:c r="I63" s="9" t="str"/>
       <x:c r="J63" s="9" t="str"/>
       <x:c r="K63" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -34139,7 +34139,7 @@
       <x:c r="I64" s="9" t="str"/>
       <x:c r="J64" s="9" t="str"/>
       <x:c r="K64" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -34168,7 +34168,7 @@
       <x:c r="I65" s="9" t="str"/>
       <x:c r="J65" s="9" t="str"/>
       <x:c r="K65" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -34197,7 +34197,7 @@
       <x:c r="I66" s="9" t="str"/>
       <x:c r="J66" s="9" t="str"/>
       <x:c r="K66" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -34228,7 +34228,7 @@
       </x:c>
       <x:c r="J67" s="9" t="str"/>
       <x:c r="K67" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -34257,7 +34257,7 @@
       <x:c r="I68" s="9" t="str"/>
       <x:c r="J68" s="9" t="str"/>
       <x:c r="K68" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -34282,7 +34282,7 @@
       <x:c r="I69" s="9" t="str"/>
       <x:c r="J69" s="9" t="str"/>
       <x:c r="K69" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -34309,7 +34309,7 @@
       <x:c r="I70" s="9" t="str"/>
       <x:c r="J70" s="9" t="str"/>
       <x:c r="K70" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -34334,7 +34334,7 @@
       <x:c r="I71" s="9" t="str"/>
       <x:c r="J71" s="9" t="str"/>
       <x:c r="K71" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -34361,7 +34361,7 @@
       <x:c r="I72" s="9" t="str"/>
       <x:c r="J72" s="9" t="str"/>
       <x:c r="K72" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -34386,7 +34386,7 @@
       <x:c r="I73" s="9" t="str"/>
       <x:c r="J73" s="9" t="str"/>
       <x:c r="K73" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -34415,7 +34415,7 @@
       <x:c r="I74" s="9" t="str"/>
       <x:c r="J74" s="9" t="str"/>
       <x:c r="K74" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -34442,7 +34442,7 @@
       <x:c r="I75" s="9" t="str"/>
       <x:c r="J75" s="9" t="str"/>
       <x:c r="K75" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -34471,7 +34471,7 @@
       <x:c r="I76" s="9" t="str"/>
       <x:c r="J76" s="9" t="str"/>
       <x:c r="K76" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -34498,7 +34498,7 @@
       <x:c r="I77" s="9" t="str"/>
       <x:c r="J77" s="9" t="str"/>
       <x:c r="K77" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -34525,7 +34525,7 @@
       <x:c r="I78" s="9" t="str"/>
       <x:c r="J78" s="9" t="str"/>
       <x:c r="K78" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -34550,7 +34550,7 @@
       <x:c r="I79" s="9" t="str"/>
       <x:c r="J79" s="9" t="str"/>
       <x:c r="K79" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -34579,7 +34579,7 @@
       <x:c r="I80" s="9" t="str"/>
       <x:c r="J80" s="9" t="str"/>
       <x:c r="K80" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -34608,7 +34608,7 @@
       <x:c r="I81" s="9" t="str"/>
       <x:c r="J81" s="9" t="str"/>
       <x:c r="K81" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -34637,7 +34637,7 @@
       <x:c r="I82" s="9" t="str"/>
       <x:c r="J82" s="9" t="str"/>
       <x:c r="K82" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
@@ -34666,7 +34666,7 @@
       <x:c r="I83" s="9" t="str"/>
       <x:c r="J83" s="9" t="str"/>
       <x:c r="K83" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
@@ -34693,7 +34693,7 @@
       <x:c r="I84" s="9" t="str"/>
       <x:c r="J84" s="9" t="str"/>
       <x:c r="K84" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -34720,7 +34720,7 @@
       <x:c r="I85" s="9" t="str"/>
       <x:c r="J85" s="9" t="str"/>
       <x:c r="K85" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -34747,7 +34747,7 @@
       <x:c r="I86" s="9" t="str"/>
       <x:c r="J86" s="9" t="str"/>
       <x:c r="K86" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -34772,7 +34772,7 @@
       <x:c r="I87" s="9" t="str"/>
       <x:c r="J87" s="9" t="str"/>
       <x:c r="K87" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -34799,7 +34799,7 @@
       <x:c r="I88" s="9" t="str"/>
       <x:c r="J88" s="9" t="str"/>
       <x:c r="K88" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -34826,7 +34826,7 @@
       <x:c r="I89" s="9" t="str"/>
       <x:c r="J89" s="9" t="str"/>
       <x:c r="K89" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -34853,7 +34853,7 @@
       <x:c r="I90" s="9" t="str"/>
       <x:c r="J90" s="9" t="str"/>
       <x:c r="K90" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -34880,7 +34880,7 @@
       <x:c r="I91" s="9" t="str"/>
       <x:c r="J91" s="9" t="str"/>
       <x:c r="K91" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -34907,7 +34907,7 @@
       <x:c r="I92" s="9" t="str"/>
       <x:c r="J92" s="9" t="str"/>
       <x:c r="K92" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -34934,7 +34934,7 @@
       <x:c r="I93" s="9" t="str"/>
       <x:c r="J93" s="9" t="str"/>
       <x:c r="K93" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -34961,7 +34961,7 @@
       <x:c r="I94" s="9" t="str"/>
       <x:c r="J94" s="9" t="str"/>
       <x:c r="K94" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -34988,7 +34988,7 @@
       <x:c r="I95" s="9" t="str"/>
       <x:c r="J95" s="9" t="str"/>
       <x:c r="K95" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -35015,7 +35015,7 @@
       <x:c r="I96" s="9" t="str"/>
       <x:c r="J96" s="9" t="str"/>
       <x:c r="K96" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
@@ -35044,7 +35044,7 @@
       <x:c r="I97" s="9" t="str"/>
       <x:c r="J97" s="9" t="str"/>
       <x:c r="K97" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -35073,7 +35073,7 @@
       <x:c r="I98" s="9" t="str"/>
       <x:c r="J98" s="9" t="str"/>
       <x:c r="K98" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
@@ -35102,7 +35102,7 @@
       <x:c r="I99" s="9" t="str"/>
       <x:c r="J99" s="9" t="str"/>
       <x:c r="K99" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
@@ -35131,7 +35131,7 @@
       </x:c>
       <x:c r="J100" s="9" t="str"/>
       <x:c r="K100" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
@@ -35158,7 +35158,7 @@
       <x:c r="I101" s="9" t="str"/>
       <x:c r="J101" s="9" t="str"/>
       <x:c r="K101" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
@@ -35185,7 +35185,7 @@
       <x:c r="I102" s="9" t="str"/>
       <x:c r="J102" s="9" t="str"/>
       <x:c r="K102" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
@@ -35212,7 +35212,7 @@
       <x:c r="I103" s="9" t="str"/>
       <x:c r="J103" s="9" t="str"/>
       <x:c r="K103" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
@@ -35239,7 +35239,7 @@
       <x:c r="I104" s="9" t="str"/>
       <x:c r="J104" s="9" t="str"/>
       <x:c r="K104" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
@@ -35266,7 +35266,7 @@
       <x:c r="I105" s="9" t="str"/>
       <x:c r="J105" s="9" t="str"/>
       <x:c r="K105" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="106">
@@ -35295,7 +35295,7 @@
       <x:c r="I106" s="9" t="str"/>
       <x:c r="J106" s="9" t="str"/>
       <x:c r="K106" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="107">
@@ -35322,7 +35322,7 @@
       <x:c r="I107" s="9" t="str"/>
       <x:c r="J107" s="9" t="str"/>
       <x:c r="K107" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
@@ -35349,7 +35349,7 @@
       <x:c r="I108" s="9" t="str"/>
       <x:c r="J108" s="9" t="str"/>
       <x:c r="K108" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
@@ -35376,7 +35376,7 @@
       <x:c r="I109" s="9" t="str"/>
       <x:c r="J109" s="9" t="str"/>
       <x:c r="K109" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
@@ -35403,7 +35403,7 @@
       <x:c r="I110" s="9" t="str"/>
       <x:c r="J110" s="9" t="str"/>
       <x:c r="K110" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
@@ -35432,7 +35432,7 @@
       <x:c r="I111" s="9" t="str"/>
       <x:c r="J111" s="9" t="str"/>
       <x:c r="K111" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
@@ -35459,7 +35459,7 @@
       <x:c r="I112" s="9" t="str"/>
       <x:c r="J112" s="9" t="str"/>
       <x:c r="K112" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
@@ -35488,7 +35488,7 @@
       </x:c>
       <x:c r="J113" s="9" t="str"/>
       <x:c r="K113" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -35517,7 +35517,7 @@
       </x:c>
       <x:c r="J114" s="9" t="str"/>
       <x:c r="K114" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
@@ -35546,7 +35546,7 @@
       </x:c>
       <x:c r="J115" s="9" t="str"/>
       <x:c r="K115" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
@@ -35575,7 +35575,7 @@
       </x:c>
       <x:c r="J116" s="9" t="str"/>
       <x:c r="K116" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
@@ -35606,7 +35606,7 @@
       </x:c>
       <x:c r="J117" s="9" t="str"/>
       <x:c r="K117" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
@@ -35635,7 +35635,7 @@
       </x:c>
       <x:c r="J118" s="9" t="str"/>
       <x:c r="K118" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
@@ -35664,7 +35664,7 @@
       </x:c>
       <x:c r="J119" s="9" t="str"/>
       <x:c r="K119" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
@@ -35691,7 +35691,7 @@
       <x:c r="I120" s="9" t="str"/>
       <x:c r="J120" s="9" t="str"/>
       <x:c r="K120" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
@@ -35722,7 +35722,7 @@
       </x:c>
       <x:c r="J121" s="9" t="str"/>
       <x:c r="K121" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
@@ -35753,7 +35753,7 @@
       </x:c>
       <x:c r="J122" s="9" t="str"/>
       <x:c r="K122" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
@@ -35784,7 +35784,7 @@
       </x:c>
       <x:c r="J123" s="9" t="str"/>
       <x:c r="K123" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
@@ -35815,7 +35815,7 @@
       </x:c>
       <x:c r="J124" s="9" t="str"/>
       <x:c r="K124" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
@@ -35846,7 +35846,7 @@
       </x:c>
       <x:c r="J125" s="9" t="str"/>
       <x:c r="K125" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
@@ -35875,7 +35875,7 @@
       </x:c>
       <x:c r="J126" s="9" t="str"/>
       <x:c r="K126" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
@@ -35904,7 +35904,7 @@
       </x:c>
       <x:c r="J127" s="9" t="str"/>
       <x:c r="K127" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
@@ -35931,7 +35931,7 @@
       </x:c>
       <x:c r="J128" s="9" t="str"/>
       <x:c r="K128" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
@@ -35962,7 +35962,7 @@
       </x:c>
       <x:c r="J129" s="9" t="str"/>
       <x:c r="K129" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
@@ -35991,7 +35991,7 @@
       </x:c>
       <x:c r="J130" s="9" t="str"/>
       <x:c r="K130" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
@@ -36020,7 +36020,7 @@
       </x:c>
       <x:c r="J131" s="9" t="str"/>
       <x:c r="K131" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
@@ -36049,7 +36049,7 @@
       </x:c>
       <x:c r="J132" s="9" t="str"/>
       <x:c r="K132" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
@@ -36080,7 +36080,7 @@
       </x:c>
       <x:c r="J133" s="9" t="str"/>
       <x:c r="K133" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
@@ -36111,7 +36111,7 @@
       </x:c>
       <x:c r="J134" s="9" t="str"/>
       <x:c r="K134" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
@@ -36142,7 +36142,7 @@
       </x:c>
       <x:c r="J135" s="9" t="str"/>
       <x:c r="K135" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
@@ -36173,7 +36173,7 @@
       </x:c>
       <x:c r="J136" s="9" t="str"/>
       <x:c r="K136" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
@@ -36204,7 +36204,7 @@
       </x:c>
       <x:c r="J137" s="9" t="str"/>
       <x:c r="K137" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="138">
@@ -36235,7 +36235,7 @@
       </x:c>
       <x:c r="J138" s="9" t="str"/>
       <x:c r="K138" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="139">
@@ -36266,7 +36266,7 @@
       </x:c>
       <x:c r="J139" s="9" t="str"/>
       <x:c r="K139" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="140">
@@ -36297,7 +36297,7 @@
       </x:c>
       <x:c r="J140" s="9" t="str"/>
       <x:c r="K140" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="141">
@@ -36328,7 +36328,7 @@
       </x:c>
       <x:c r="J141" s="9" t="str"/>
       <x:c r="K141" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="142">
@@ -36359,7 +36359,7 @@
       </x:c>
       <x:c r="J142" s="9" t="str"/>
       <x:c r="K142" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="143">
@@ -36388,7 +36388,7 @@
       </x:c>
       <x:c r="J143" s="9" t="str"/>
       <x:c r="K143" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="144">
@@ -36419,7 +36419,7 @@
       </x:c>
       <x:c r="J144" s="9" t="str"/>
       <x:c r="K144" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="145">
@@ -36448,7 +36448,7 @@
       </x:c>
       <x:c r="J145" s="9" t="str"/>
       <x:c r="K145" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="146">
@@ -36477,7 +36477,7 @@
       </x:c>
       <x:c r="J146" s="9" t="str"/>
       <x:c r="K146" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="147">
@@ -36508,7 +36508,7 @@
       </x:c>
       <x:c r="J147" s="9" t="str"/>
       <x:c r="K147" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="148">
@@ -36537,7 +36537,7 @@
       </x:c>
       <x:c r="J148" s="9" t="str"/>
       <x:c r="K148" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="149">
@@ -36566,7 +36566,7 @@
       </x:c>
       <x:c r="J149" s="9" t="str"/>
       <x:c r="K149" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="150">
@@ -36595,7 +36595,7 @@
       </x:c>
       <x:c r="J150" s="9" t="str"/>
       <x:c r="K150" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="151">
@@ -36624,7 +36624,7 @@
       </x:c>
       <x:c r="J151" s="9" t="str"/>
       <x:c r="K151" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="152">
@@ -36653,7 +36653,7 @@
       </x:c>
       <x:c r="J152" s="9" t="str"/>
       <x:c r="K152" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="153">
@@ -36682,7 +36682,7 @@
       </x:c>
       <x:c r="J153" s="9" t="str"/>
       <x:c r="K153" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="154">
@@ -36713,7 +36713,7 @@
       </x:c>
       <x:c r="J154" s="9" t="str"/>
       <x:c r="K154" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="155">
@@ -36740,7 +36740,7 @@
       <x:c r="I155" s="9" t="str"/>
       <x:c r="J155" s="9" t="str"/>
       <x:c r="K155" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="156">
@@ -36769,7 +36769,7 @@
       <x:c r="I156" s="9" t="str"/>
       <x:c r="J156" s="9" t="str"/>
       <x:c r="K156" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="157">
@@ -36796,7 +36796,7 @@
       <x:c r="I157" s="9" t="str"/>
       <x:c r="J157" s="9" t="str"/>
       <x:c r="K157" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="158">
@@ -36823,7 +36823,7 @@
       <x:c r="I158" s="9" t="str"/>
       <x:c r="J158" s="9" t="str"/>
       <x:c r="K158" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="159">
@@ -36850,7 +36850,7 @@
       <x:c r="I159" s="9" t="str"/>
       <x:c r="J159" s="9" t="str"/>
       <x:c r="K159" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="160">
@@ -36877,7 +36877,7 @@
       <x:c r="I160" s="9" t="str"/>
       <x:c r="J160" s="9" t="str"/>
       <x:c r="K160" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="161">
@@ -36906,7 +36906,7 @@
       <x:c r="I161" s="9" t="str"/>
       <x:c r="J161" s="9" t="str"/>
       <x:c r="K161" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="162">
@@ -36935,7 +36935,7 @@
       <x:c r="I162" s="9" t="str"/>
       <x:c r="J162" s="9" t="str"/>
       <x:c r="K162" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="163">
@@ -36962,7 +36962,7 @@
       <x:c r="I163" s="9" t="str"/>
       <x:c r="J163" s="9" t="str"/>
       <x:c r="K163" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="164">
@@ -36989,7 +36989,7 @@
       <x:c r="I164" s="9" t="str"/>
       <x:c r="J164" s="9" t="str"/>
       <x:c r="K164" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="165">
@@ -37016,7 +37016,7 @@
       <x:c r="I165" s="9" t="str"/>
       <x:c r="J165" s="9" t="str"/>
       <x:c r="K165" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="166">
@@ -37043,7 +37043,7 @@
       <x:c r="I166" s="9" t="str"/>
       <x:c r="J166" s="9" t="str"/>
       <x:c r="K166" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="167">
@@ -37070,7 +37070,7 @@
       <x:c r="I167" s="9" t="str"/>
       <x:c r="J167" s="9" t="str"/>
       <x:c r="K167" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="168">
@@ -37099,7 +37099,7 @@
       <x:c r="I168" s="9" t="str"/>
       <x:c r="J168" s="9" t="str"/>
       <x:c r="K168" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="169">
@@ -37128,7 +37128,7 @@
       <x:c r="I169" s="9" t="str"/>
       <x:c r="J169" s="9" t="str"/>
       <x:c r="K169" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="170">
@@ -37157,7 +37157,7 @@
       <x:c r="I170" s="9" t="str"/>
       <x:c r="J170" s="9" t="str"/>
       <x:c r="K170" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="171">
@@ -37184,7 +37184,7 @@
       <x:c r="I171" s="9" t="str"/>
       <x:c r="J171" s="9" t="str"/>
       <x:c r="K171" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="172">
@@ -37211,7 +37211,7 @@
       <x:c r="I172" s="9" t="str"/>
       <x:c r="J172" s="9" t="str"/>
       <x:c r="K172" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="173">
@@ -37238,7 +37238,7 @@
       <x:c r="I173" s="9" t="str"/>
       <x:c r="J173" s="9" t="str"/>
       <x:c r="K173" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="174">
@@ -37265,7 +37265,7 @@
       <x:c r="I174" s="9" t="str"/>
       <x:c r="J174" s="9" t="str"/>
       <x:c r="K174" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="175">
@@ -37292,7 +37292,7 @@
       <x:c r="I175" s="9" t="str"/>
       <x:c r="J175" s="9" t="str"/>
       <x:c r="K175" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="176">
@@ -37319,7 +37319,7 @@
       <x:c r="I176" s="9" t="str"/>
       <x:c r="J176" s="9" t="str"/>
       <x:c r="K176" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="177">
@@ -37346,7 +37346,7 @@
       <x:c r="I177" s="9" t="str"/>
       <x:c r="J177" s="9" t="str"/>
       <x:c r="K177" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="178">
@@ -37375,7 +37375,7 @@
       <x:c r="I178" s="9" t="str"/>
       <x:c r="J178" s="9" t="str"/>
       <x:c r="K178" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="179">
@@ -37404,7 +37404,7 @@
       <x:c r="I179" s="9" t="str"/>
       <x:c r="J179" s="9" t="str"/>
       <x:c r="K179" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="180">
@@ -37433,7 +37433,7 @@
       <x:c r="I180" s="9" t="str"/>
       <x:c r="J180" s="9" t="str"/>
       <x:c r="K180" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="181">
@@ -37462,7 +37462,7 @@
       <x:c r="I181" s="9" t="str"/>
       <x:c r="J181" s="9" t="str"/>
       <x:c r="K181" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -37491,7 +37491,7 @@
       <x:c r="I182" s="9" t="str"/>
       <x:c r="J182" s="9" t="str"/>
       <x:c r="K182" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="183">
@@ -37522,7 +37522,7 @@
       </x:c>
       <x:c r="J183" s="9" t="str"/>
       <x:c r="K183" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="184">
@@ -37551,7 +37551,7 @@
       <x:c r="I184" s="9" t="str"/>
       <x:c r="J184" s="9" t="str"/>
       <x:c r="K184" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="185">
@@ -37578,7 +37578,7 @@
       </x:c>
       <x:c r="J185" s="9" t="str"/>
       <x:c r="K185" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="186">
@@ -37607,7 +37607,7 @@
       <x:c r="I186" s="9" t="str"/>
       <x:c r="J186" s="9" t="str"/>
       <x:c r="K186" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="187">
@@ -37638,7 +37638,7 @@
       </x:c>
       <x:c r="J187" s="9" t="str"/>
       <x:c r="K187" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="188">
@@ -37667,7 +37667,7 @@
       <x:c r="I188" s="9" t="str"/>
       <x:c r="J188" s="9" t="str"/>
       <x:c r="K188" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="189">
@@ -37694,7 +37694,7 @@
       </x:c>
       <x:c r="J189" s="9" t="str"/>
       <x:c r="K189" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="190">
@@ -37725,7 +37725,7 @@
       </x:c>
       <x:c r="J190" s="9" t="str"/>
       <x:c r="K190" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="191">
@@ -37756,7 +37756,7 @@
       </x:c>
       <x:c r="J191" s="9" t="str"/>
       <x:c r="K191" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="192">
@@ -37785,7 +37785,7 @@
       </x:c>
       <x:c r="J192" s="9" t="str"/>
       <x:c r="K192" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="193">
@@ -37814,7 +37814,7 @@
       <x:c r="I193" s="9" t="str"/>
       <x:c r="J193" s="9" t="str"/>
       <x:c r="K193" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="194">
@@ -37845,7 +37845,7 @@
       </x:c>
       <x:c r="J194" s="9" t="str"/>
       <x:c r="K194" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="195">
@@ -37876,7 +37876,7 @@
       </x:c>
       <x:c r="J195" s="9" t="str"/>
       <x:c r="K195" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="196">
@@ -37905,7 +37905,7 @@
       </x:c>
       <x:c r="J196" s="9" t="str"/>
       <x:c r="K196" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="197">
@@ -37934,7 +37934,7 @@
       <x:c r="I197" s="9" t="str"/>
       <x:c r="J197" s="9" t="str"/>
       <x:c r="K197" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="198">
@@ -37965,7 +37965,7 @@
       </x:c>
       <x:c r="J198" s="9" t="str"/>
       <x:c r="K198" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="199">
@@ -37994,7 +37994,7 @@
       <x:c r="I199" s="9" t="str"/>
       <x:c r="J199" s="9" t="str"/>
       <x:c r="K199" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="200">
@@ -38025,7 +38025,7 @@
       </x:c>
       <x:c r="J200" s="9" t="str"/>
       <x:c r="K200" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="201">
@@ -38054,7 +38054,7 @@
       <x:c r="I201" s="9" t="str"/>
       <x:c r="J201" s="9" t="str"/>
       <x:c r="K201" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="202">
@@ -38083,7 +38083,7 @@
       <x:c r="I202" s="9" t="str"/>
       <x:c r="J202" s="9" t="str"/>
       <x:c r="K202" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="203">
@@ -38110,7 +38110,7 @@
       <x:c r="I203" s="9" t="str"/>
       <x:c r="J203" s="9" t="str"/>
       <x:c r="K203" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="204">
@@ -38135,7 +38135,7 @@
       <x:c r="I204" s="9" t="str"/>
       <x:c r="J204" s="9" t="str"/>
       <x:c r="K204" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="205">
@@ -38162,7 +38162,7 @@
       <x:c r="I205" s="9" t="str"/>
       <x:c r="J205" s="9" t="str"/>
       <x:c r="K205" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="206">
@@ -38189,7 +38189,7 @@
       <x:c r="I206" s="9" t="str"/>
       <x:c r="J206" s="9" t="str"/>
       <x:c r="K206" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="207">
@@ -38216,7 +38216,7 @@
       <x:c r="I207" s="9" t="str"/>
       <x:c r="J207" s="9" t="str"/>
       <x:c r="K207" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="208">
@@ -38243,7 +38243,7 @@
       <x:c r="I208" s="9" t="str"/>
       <x:c r="J208" s="9" t="str"/>
       <x:c r="K208" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="209">
@@ -38270,7 +38270,7 @@
       <x:c r="I209" s="9" t="str"/>
       <x:c r="J209" s="9" t="str"/>
       <x:c r="K209" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="210">
@@ -38299,7 +38299,7 @@
       <x:c r="I210" s="9" t="str"/>
       <x:c r="J210" s="9" t="str"/>
       <x:c r="K210" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="211">
@@ -38328,7 +38328,7 @@
       <x:c r="I211" s="9" t="str"/>
       <x:c r="J211" s="9" t="str"/>
       <x:c r="K211" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="212">
@@ -38357,7 +38357,7 @@
       <x:c r="I212" s="9" t="str"/>
       <x:c r="J212" s="9" t="str"/>
       <x:c r="K212" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="213">
@@ -38384,7 +38384,7 @@
       <x:c r="I213" s="9" t="str"/>
       <x:c r="J213" s="9" t="str"/>
       <x:c r="K213" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="214">
@@ -38411,7 +38411,7 @@
       <x:c r="I214" s="9" t="str"/>
       <x:c r="J214" s="9" t="str"/>
       <x:c r="K214" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="215">
@@ -38442,7 +38442,7 @@
       </x:c>
       <x:c r="J215" s="9" t="str"/>
       <x:c r="K215" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="216">
@@ -38469,7 +38469,7 @@
       <x:c r="I216" s="9" t="str"/>
       <x:c r="J216" s="9" t="str"/>
       <x:c r="K216" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="217">
@@ -38498,7 +38498,7 @@
       <x:c r="I217" s="9" t="str"/>
       <x:c r="J217" s="9" t="str"/>
       <x:c r="K217" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="218">
@@ -38525,7 +38525,7 @@
       <x:c r="I218" s="9" t="str"/>
       <x:c r="J218" s="9" t="str"/>
       <x:c r="K218" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="219">
@@ -38556,7 +38556,7 @@
       </x:c>
       <x:c r="J219" s="9" t="str"/>
       <x:c r="K219" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="220">
@@ -38581,7 +38581,7 @@
       <x:c r="I220" s="9" t="str"/>
       <x:c r="J220" s="9" t="str"/>
       <x:c r="K220" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="221">
@@ -38608,7 +38608,7 @@
       <x:c r="I221" s="9" t="str"/>
       <x:c r="J221" s="9" t="str"/>
       <x:c r="K221" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="222">
@@ -38635,7 +38635,7 @@
       <x:c r="I222" s="9" t="str"/>
       <x:c r="J222" s="9" t="str"/>
       <x:c r="K222" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="223">
@@ -38662,7 +38662,7 @@
       <x:c r="I223" s="9" t="str"/>
       <x:c r="J223" s="9" t="str"/>
       <x:c r="K223" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="224">
@@ -38689,7 +38689,7 @@
       <x:c r="I224" s="9" t="str"/>
       <x:c r="J224" s="9" t="str"/>
       <x:c r="K224" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="225">
@@ -38716,7 +38716,7 @@
       <x:c r="I225" s="9" t="str"/>
       <x:c r="J225" s="9" t="str"/>
       <x:c r="K225" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="226">
@@ -38745,7 +38745,7 @@
       <x:c r="I226" s="9" t="str"/>
       <x:c r="J226" s="9" t="str"/>
       <x:c r="K226" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="227">
@@ -38772,7 +38772,7 @@
       <x:c r="I227" s="9" t="str"/>
       <x:c r="J227" s="9" t="str"/>
       <x:c r="K227" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="228">
@@ -38797,7 +38797,7 @@
       <x:c r="I228" s="9" t="str"/>
       <x:c r="J228" s="9" t="str"/>
       <x:c r="K228" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="229">
@@ -38824,7 +38824,7 @@
       <x:c r="I229" s="9" t="str"/>
       <x:c r="J229" s="9" t="str"/>
       <x:c r="K229" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="230">
@@ -38851,7 +38851,7 @@
       <x:c r="I230" s="9" t="str"/>
       <x:c r="J230" s="9" t="str"/>
       <x:c r="K230" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="231">
@@ -38878,7 +38878,7 @@
       <x:c r="I231" s="9" t="str"/>
       <x:c r="J231" s="9" t="str"/>
       <x:c r="K231" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="232">
@@ -38905,7 +38905,7 @@
       <x:c r="I232" s="9" t="str"/>
       <x:c r="J232" s="9" t="str"/>
       <x:c r="K232" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="233">
@@ -38932,7 +38932,7 @@
       <x:c r="I233" s="9" t="str"/>
       <x:c r="J233" s="9" t="str"/>
       <x:c r="K233" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="234">
@@ -38961,7 +38961,7 @@
       </x:c>
       <x:c r="J234" s="9" t="str"/>
       <x:c r="K234" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="235">
@@ -38988,7 +38988,7 @@
       <x:c r="I235" s="9" t="str"/>
       <x:c r="J235" s="9" t="str"/>
       <x:c r="K235" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="236">
@@ -39015,7 +39015,7 @@
       <x:c r="I236" s="9" t="str"/>
       <x:c r="J236" s="9" t="str"/>
       <x:c r="K236" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="237">
@@ -39042,7 +39042,7 @@
       <x:c r="I237" s="9" t="str"/>
       <x:c r="J237" s="9" t="str"/>
       <x:c r="K237" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="238">
@@ -39071,7 +39071,7 @@
       </x:c>
       <x:c r="J238" s="9" t="str"/>
       <x:c r="K238" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="239">
@@ -39098,7 +39098,7 @@
       <x:c r="I239" s="9" t="str"/>
       <x:c r="J239" s="9" t="str"/>
       <x:c r="K239" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="240">
@@ -39125,7 +39125,7 @@
       <x:c r="I240" s="9" t="str"/>
       <x:c r="J240" s="9" t="str"/>
       <x:c r="K240" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="241">
@@ -39152,7 +39152,7 @@
       <x:c r="I241" s="9" t="str"/>
       <x:c r="J241" s="9" t="str"/>
       <x:c r="K241" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="242">
@@ -39181,7 +39181,7 @@
       </x:c>
       <x:c r="J242" s="9" t="str"/>
       <x:c r="K242" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="243">
@@ -39210,7 +39210,7 @@
       </x:c>
       <x:c r="J243" s="9" t="str"/>
       <x:c r="K243" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="244">
@@ -39239,7 +39239,7 @@
       </x:c>
       <x:c r="J244" s="9" t="str"/>
       <x:c r="K244" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="245">
@@ -39268,7 +39268,7 @@
       <x:c r="I245" s="9" t="str"/>
       <x:c r="J245" s="9" t="str"/>
       <x:c r="K245" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="246">
@@ -39295,7 +39295,7 @@
       <x:c r="I246" s="9" t="str"/>
       <x:c r="J246" s="9" t="str"/>
       <x:c r="K246" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="247">
@@ -39326,7 +39326,7 @@
       </x:c>
       <x:c r="J247" s="9" t="str"/>
       <x:c r="K247" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="248">
@@ -39353,7 +39353,7 @@
       </x:c>
       <x:c r="J248" s="9" t="str"/>
       <x:c r="K248" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="249">
@@ -39382,7 +39382,7 @@
       <x:c r="I249" s="9" t="str"/>
       <x:c r="J249" s="9" t="str"/>
       <x:c r="K249" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="250">
@@ -39411,7 +39411,7 @@
       <x:c r="I250" s="9" t="str"/>
       <x:c r="J250" s="9" t="str"/>
       <x:c r="K250" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="251">
@@ -39440,7 +39440,7 @@
       <x:c r="I251" s="9" t="str"/>
       <x:c r="J251" s="9" t="str"/>
       <x:c r="K251" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="252">
@@ -39469,7 +39469,7 @@
       <x:c r="I252" s="9" t="str"/>
       <x:c r="J252" s="9" t="str"/>
       <x:c r="K252" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="253">
@@ -39498,7 +39498,7 @@
       <x:c r="I253" s="9" t="str"/>
       <x:c r="J253" s="9" t="str"/>
       <x:c r="K253" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="254">
@@ -39527,7 +39527,7 @@
       <x:c r="I254" s="9" t="str"/>
       <x:c r="J254" s="9" t="str"/>
       <x:c r="K254" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="255">
@@ -39556,7 +39556,7 @@
       <x:c r="I255" s="9" t="str"/>
       <x:c r="J255" s="9" t="str"/>
       <x:c r="K255" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="256">
@@ -39585,7 +39585,7 @@
       <x:c r="I256" s="9" t="str"/>
       <x:c r="J256" s="9" t="str"/>
       <x:c r="K256" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="257">
@@ -39616,7 +39616,7 @@
       </x:c>
       <x:c r="J257" s="9" t="str"/>
       <x:c r="K257" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="258">
@@ -39647,7 +39647,7 @@
       </x:c>
       <x:c r="J258" s="9" t="str"/>
       <x:c r="K258" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="259">
@@ -39674,7 +39674,7 @@
       <x:c r="I259" s="9" t="str"/>
       <x:c r="J259" s="9" t="str"/>
       <x:c r="K259" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="260">
@@ -39701,7 +39701,7 @@
       <x:c r="I260" s="9" t="str"/>
       <x:c r="J260" s="9" t="str"/>
       <x:c r="K260" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="261">
@@ -39728,7 +39728,7 @@
       <x:c r="I261" s="9" t="str"/>
       <x:c r="J261" s="9" t="str"/>
       <x:c r="K261" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="262">
@@ -39755,7 +39755,7 @@
       <x:c r="I262" s="9" t="str"/>
       <x:c r="J262" s="9" t="str"/>
       <x:c r="K262" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="263">
@@ -39782,7 +39782,7 @@
       <x:c r="I263" s="9" t="str"/>
       <x:c r="J263" s="9" t="str"/>
       <x:c r="K263" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="264">
@@ -39809,7 +39809,7 @@
       <x:c r="I264" s="9" t="str"/>
       <x:c r="J264" s="9" t="str"/>
       <x:c r="K264" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="265">
@@ -39836,7 +39836,7 @@
       <x:c r="I265" s="9" t="str"/>
       <x:c r="J265" s="9" t="str"/>
       <x:c r="K265" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="266">
@@ -39863,7 +39863,7 @@
       <x:c r="I266" s="9" t="str"/>
       <x:c r="J266" s="9" t="str"/>
       <x:c r="K266" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="267">
@@ -39890,7 +39890,7 @@
       <x:c r="I267" s="9" t="str"/>
       <x:c r="J267" s="9" t="str"/>
       <x:c r="K267" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="268">
@@ -39917,7 +39917,7 @@
       <x:c r="I268" s="9" t="str"/>
       <x:c r="J268" s="9" t="str"/>
       <x:c r="K268" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="269">
@@ -39944,7 +39944,7 @@
       <x:c r="I269" s="9" t="str"/>
       <x:c r="J269" s="9" t="str"/>
       <x:c r="K269" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="270">
@@ -39971,7 +39971,7 @@
       <x:c r="I270" s="9" t="str"/>
       <x:c r="J270" s="9" t="str"/>
       <x:c r="K270" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="271">
@@ -39998,7 +39998,7 @@
       <x:c r="I271" s="9" t="str"/>
       <x:c r="J271" s="9" t="str"/>
       <x:c r="K271" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="272">
@@ -40025,7 +40025,7 @@
       <x:c r="I272" s="9" t="str"/>
       <x:c r="J272" s="9" t="str"/>
       <x:c r="K272" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="273">
@@ -40054,7 +40054,7 @@
       <x:c r="I273" s="9" t="str"/>
       <x:c r="J273" s="9" t="str"/>
       <x:c r="K273" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="274">
@@ -40081,7 +40081,7 @@
       <x:c r="I274" s="9" t="str"/>
       <x:c r="J274" s="9" t="str"/>
       <x:c r="K274" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="275">
@@ -40108,7 +40108,7 @@
       <x:c r="I275" s="9" t="str"/>
       <x:c r="J275" s="9" t="str"/>
       <x:c r="K275" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="276">
@@ -40135,7 +40135,7 @@
       <x:c r="I276" s="9" t="str"/>
       <x:c r="J276" s="9" t="str"/>
       <x:c r="K276" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="277">
@@ -40164,7 +40164,7 @@
       <x:c r="I277" s="9" t="str"/>
       <x:c r="J277" s="9" t="str"/>
       <x:c r="K277" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="278">
@@ -40191,7 +40191,7 @@
       <x:c r="I278" s="9" t="str"/>
       <x:c r="J278" s="9" t="str"/>
       <x:c r="K278" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="279">
@@ -40218,7 +40218,7 @@
       <x:c r="I279" s="9" t="str"/>
       <x:c r="J279" s="9" t="str"/>
       <x:c r="K279" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="280">
@@ -40245,7 +40245,7 @@
       <x:c r="I280" s="9" t="str"/>
       <x:c r="J280" s="9" t="str"/>
       <x:c r="K280" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="281">
@@ -40272,7 +40272,7 @@
       <x:c r="I281" s="9" t="str"/>
       <x:c r="J281" s="9" t="str"/>
       <x:c r="K281" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="282">
@@ -40299,7 +40299,7 @@
       <x:c r="I282" s="9" t="str"/>
       <x:c r="J282" s="9" t="str"/>
       <x:c r="K282" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="283">
@@ -40326,7 +40326,7 @@
       <x:c r="I283" s="9" t="str"/>
       <x:c r="J283" s="9" t="str"/>
       <x:c r="K283" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="284">
@@ -40353,7 +40353,7 @@
       <x:c r="I284" s="9" t="str"/>
       <x:c r="J284" s="9" t="str"/>
       <x:c r="K284" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="285">
@@ -40380,7 +40380,7 @@
       <x:c r="I285" s="9" t="str"/>
       <x:c r="J285" s="9" t="str"/>
       <x:c r="K285" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="286">
@@ -40407,7 +40407,7 @@
       <x:c r="I286" s="9" t="str"/>
       <x:c r="J286" s="9" t="str"/>
       <x:c r="K286" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="287">
@@ -40434,7 +40434,7 @@
       <x:c r="I287" s="9" t="str"/>
       <x:c r="J287" s="9" t="str"/>
       <x:c r="K287" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="288">
@@ -40461,7 +40461,7 @@
       <x:c r="I288" s="9" t="str"/>
       <x:c r="J288" s="9" t="str"/>
       <x:c r="K288" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="289">
@@ -40490,7 +40490,7 @@
       <x:c r="I289" s="9" t="str"/>
       <x:c r="J289" s="9" t="str"/>
       <x:c r="K289" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="290">
@@ -40517,7 +40517,7 @@
       <x:c r="I290" s="9" t="str"/>
       <x:c r="J290" s="9" t="str"/>
       <x:c r="K290" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="291">
@@ -40544,7 +40544,7 @@
       <x:c r="I291" s="9" t="str"/>
       <x:c r="J291" s="9" t="str"/>
       <x:c r="K291" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="292">
@@ -40571,7 +40571,7 @@
       <x:c r="I292" s="9" t="str"/>
       <x:c r="J292" s="9" t="str"/>
       <x:c r="K292" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="293">
@@ -40598,7 +40598,7 @@
       <x:c r="I293" s="9" t="str"/>
       <x:c r="J293" s="9" t="str"/>
       <x:c r="K293" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="294">
@@ -40625,7 +40625,7 @@
       <x:c r="I294" s="9" t="str"/>
       <x:c r="J294" s="9" t="str"/>
       <x:c r="K294" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="295">
@@ -40652,7 +40652,7 @@
       <x:c r="I295" s="9" t="str"/>
       <x:c r="J295" s="9" t="str"/>
       <x:c r="K295" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="296">
@@ -40679,7 +40679,7 @@
       <x:c r="I296" s="9" t="str"/>
       <x:c r="J296" s="9" t="str"/>
       <x:c r="K296" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="297">
@@ -40706,7 +40706,7 @@
       <x:c r="I297" s="9" t="str"/>
       <x:c r="J297" s="9" t="str"/>
       <x:c r="K297" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="298">
@@ -40733,7 +40733,7 @@
       <x:c r="I298" s="9" t="str"/>
       <x:c r="J298" s="9" t="str"/>
       <x:c r="K298" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="299">
@@ -40760,7 +40760,7 @@
       <x:c r="I299" s="9" t="str"/>
       <x:c r="J299" s="9" t="str"/>
       <x:c r="K299" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="300">
@@ -40787,7 +40787,7 @@
       <x:c r="I300" s="9" t="str"/>
       <x:c r="J300" s="9" t="str"/>
       <x:c r="K300" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="301">
@@ -40814,7 +40814,7 @@
       <x:c r="I301" s="9" t="str"/>
       <x:c r="J301" s="9" t="str"/>
       <x:c r="K301" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="302">
@@ -40841,7 +40841,7 @@
       <x:c r="I302" s="9" t="str"/>
       <x:c r="J302" s="9" t="str"/>
       <x:c r="K302" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="303">
@@ -40868,7 +40868,7 @@
       <x:c r="I303" s="9" t="str"/>
       <x:c r="J303" s="9" t="str"/>
       <x:c r="K303" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="304">
@@ -40895,7 +40895,7 @@
       <x:c r="I304" s="9" t="str"/>
       <x:c r="J304" s="9" t="str"/>
       <x:c r="K304" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="305">
@@ -40922,7 +40922,7 @@
       <x:c r="I305" s="9" t="str"/>
       <x:c r="J305" s="9" t="str"/>
       <x:c r="K305" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="306">
@@ -40949,7 +40949,7 @@
       <x:c r="I306" s="9" t="str"/>
       <x:c r="J306" s="9" t="str"/>
       <x:c r="K306" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="307">
@@ -40976,7 +40976,7 @@
       <x:c r="I307" s="9" t="str"/>
       <x:c r="J307" s="9" t="str"/>
       <x:c r="K307" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="308">
@@ -41001,7 +41001,7 @@
       <x:c r="I308" s="9" t="str"/>
       <x:c r="J308" s="9" t="str"/>
       <x:c r="K308" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="309">
@@ -41030,7 +41030,7 @@
       </x:c>
       <x:c r="J309" s="9" t="str"/>
       <x:c r="K309" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="310">
@@ -41059,7 +41059,7 @@
       </x:c>
       <x:c r="J310" s="9" t="str"/>
       <x:c r="K310" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="311">
@@ -41086,7 +41086,7 @@
       <x:c r="I311" s="9" t="str"/>
       <x:c r="J311" s="9" t="str"/>
       <x:c r="K311" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="312">
@@ -41113,7 +41113,7 @@
       <x:c r="I312" s="9" t="str"/>
       <x:c r="J312" s="9" t="str"/>
       <x:c r="K312" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="313">
@@ -41140,7 +41140,7 @@
       <x:c r="I313" s="9" t="str"/>
       <x:c r="J313" s="9" t="str"/>
       <x:c r="K313" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="314">
@@ -41169,7 +41169,7 @@
       <x:c r="I314" s="9" t="str"/>
       <x:c r="J314" s="9" t="str"/>
       <x:c r="K314" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="315">
@@ -41198,7 +41198,7 @@
       </x:c>
       <x:c r="J315" s="9" t="str"/>
       <x:c r="K315" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="316">
@@ -41225,7 +41225,7 @@
       <x:c r="I316" s="9" t="str"/>
       <x:c r="J316" s="9" t="str"/>
       <x:c r="K316" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="317">
@@ -41252,7 +41252,7 @@
       <x:c r="I317" s="9" t="str"/>
       <x:c r="J317" s="9" t="str"/>
       <x:c r="K317" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="318">
@@ -41279,7 +41279,7 @@
       <x:c r="I318" s="9" t="str"/>
       <x:c r="J318" s="9" t="str"/>
       <x:c r="K318" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="319">
@@ -41308,7 +41308,7 @@
       </x:c>
       <x:c r="J319" s="9" t="str"/>
       <x:c r="K319" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
     <x:row r="320">
@@ -41337,13 +41337,13 @@
       </x:c>
       <x:c r="J320" s="9" t="str"/>
       <x:c r="K320" s="9" t="str">
-        <x:v>Observed values and SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
+        <x:v>Nonmissing PUF X values may include imputed values; this is not direct-response coverage. SAS availability codes only; wording/scale invariance requires questionnaire review.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66a19e693ea94bbb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fa73357fe7e46eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41354,7 +41354,7 @@
   <x:cols>
     <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="44" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="27" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="52" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="21" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
@@ -41371,7 +41371,7 @@
         <x:v>Nhãn SAS / câu hỏi</x:v>
       </x:c>
       <x:c r="C1" s="13" t="str">
-        <x:v>Wave có phản hồi quan sát</x:v>
+        <x:v>Wave có giá trị PUF không thiếu (có thể đã impute)</x:v>
       </x:c>
       <x:c r="D1" s="13" t="str">
         <x:v>Wave không được hỏi</x:v>
@@ -41551,7 +41551,7 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="I7" s="9" t="str">
-        <x:v>WORDING_VERSION_BREAK; from waves 11-12 the option changes from 'borrow enough money from a bank or credit union' to 'borrow a significant amount from a bank or credit union'; response scale labels are stable in checked PDFs; stratify/sensitivity for long-run trends</x:v>
+        <x:v>COMMON_ITEM_CANDIDATE; wording found in all packages; verify routing/respondent/mode and scale before trend use</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -41578,7 +41578,7 @@
       </x:c>
       <x:c r="H8" s="9" t="str"/>
       <x:c r="I8" s="9" t="str">
-        <x:v>Separate from x14a_1: PIMPFM scale, observed waves 7-46; do not pool raw numeric codes.</x:v>
+        <x:v>Separate from x14a_1: PIMPFM scale, nonmissing PUF values in waves 7-46; do not pool raw numeric codes.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -41605,7 +41605,7 @@
       </x:c>
       <x:c r="H9" s="9" t="str"/>
       <x:c r="I9" s="9" t="str">
-        <x:v>Separate from x14a: PVERYFM scale, observed waves 1-6; do not pool raw numeric codes.</x:v>
+        <x:v>Separate from x14a: PVERYFM scale, nonmissing PUF values in waves 1-6; do not pool raw numeric codes.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -41636,7 +41636,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde166d9d34e14c6b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R899ceeab2eac4a1d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -62380,7 +62380,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4101b047edb3434f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fefe682acae4cc3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>